<commit_message>
test: Update defect excel test file
</commit_message>
<xml_diff>
--- a/tests/domain/route_points/defect_010362.xlsx
+++ b/tests/domain/route_points/defect_010362.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hazin\Projects\bm-route-events\tests\domain\route_points\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannanazinuddin/Projects/bm-route-events/tests/domain/route_points/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DF57F2-6330-4398-B21F-C97C718C9A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A12986-F3D7-1542-BB45-4A049A290F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="22620" windowHeight="13500" tabRatio="570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>linkid</t>
   </si>
@@ -60,9 +60,6 @@
     <t>video_id</t>
   </si>
   <si>
-    <t>url_photo</t>
-  </si>
-  <si>
     <t>defects_type</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>9</t>
   </si>
   <si>
-    <t>https://123.xyz</t>
-  </si>
-  <si>
     <t>as_alg_crack</t>
   </si>
   <si>
@@ -139,6 +133,21 @@
   </si>
   <si>
     <t>as_raveling</t>
+  </si>
+  <si>
+    <t>photo_id</t>
+  </si>
+  <si>
+    <t>019d8637-6660-72be-87ec-02d0cba2ab7c</t>
+  </si>
+  <si>
+    <t>019d8637-686f-72bf-86ba-304d2be37df8</t>
+  </si>
+  <si>
+    <t>019d8637-6a02-72c0-95ba-cdd6d3f1ea8a</t>
+  </si>
+  <si>
+    <t>019d8637-6b81-72c1-9ece-38d458b4bbb7</t>
   </si>
 </sst>
 </file>
@@ -1048,28 +1057,29 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:Q6"/>
-  <sheetFormatPr defaultColWidth="17" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="17" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.83203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.5" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="3" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1796875" style="15" customWidth="1"/>
-    <col min="8" max="9" width="17" style="1"/>
-    <col min="10" max="10" width="17.453125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="16.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.1640625" style="15" customWidth="1"/>
+    <col min="8" max="8" width="17" style="1"/>
+    <col min="9" max="9" width="34.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" style="2" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="17" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1095,36 +1105,36 @@
         <v>7</v>
       </c>
       <c r="I1" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="N1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="O1" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="Q1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="10" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
@@ -1136,29 +1146,29 @@
         <v>2.8316146</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>18</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K2" s="4">
         <v>20</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N2" s="5">
         <v>2018</v>
@@ -1173,9 +1183,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3">
         <v>10</v>
@@ -1187,29 +1197,29 @@
         <v>2.8316146</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="8" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K3" s="4">
         <v>20</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N3" s="5">
         <v>2018</v>
@@ -1224,9 +1234,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B4" s="3">
         <v>10</v>
@@ -1238,29 +1248,29 @@
         <v>2.8316146</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="8" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K4" s="4">
         <v>20</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N4" s="5">
         <v>2018</v>
@@ -1275,9 +1285,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3">
         <v>10</v>
@@ -1289,29 +1299,29 @@
         <v>2.8316146</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="8" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K5" s="4">
         <v>20</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N5" s="5">
         <v>2018</v>
@@ -1326,16 +1336,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{357AB051-F3E2-47CD-8274-B6544953D183}"/>
-    <hyperlink ref="I3:I5" r:id="rId2" display="https://123.xyz" xr:uid="{95713E74-9CA5-46E4-99E9-BD04DDE5FFD1}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>